<commit_message>
Add GEG performance dashboard with charts and KPI scored table
New sheet C12 GEG Dashboard: KPI tiles vs budget, monthly charts for
revenue, EBITDA, production, stripping ratio, cash cost vs ASP and fuel
ratio, YTD cost structure, KPI score by perspective, status counts, and a
KPI scored table linked to the scorecard. Driven by the report-month
selector in C1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019cy6heYZTs4S4dMR3vbYtW
</commit_message>
<xml_diff>
--- a/docs/fpa-global-energy-group/GEG_FPA_Coal_Mining_Template.xlsx
+++ b/docs/fpa-global-energy-group/GEG_FPA_Coal_Mining_Template.xlsx
@@ -29,6 +29,7 @@
     <sheet name="C9 GEG Lap Ops" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="C10 GEG COP" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="C11 GEG KPI Scorecard" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="C12 GEG Dashboard" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46,7 +47,7 @@
     <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;;(0.00&quot;x&quot;);&quot;-&quot;"/>
     <numFmt numFmtId="170" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -142,6 +143,29 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="0052514E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000B0B0B"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0052514E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000B0B0B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="10"/>
     </font>
@@ -152,7 +176,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -189,6 +213,11 @@
         <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F3EF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -207,15 +236,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -331,11 +360,29 @@
     <xf numFmtId="168" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="17" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="17" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -371,6 +418,26 @@
           <fgColor rgb="00FFEB9C"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="00BFBDB6"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -443,6 +510,1577 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Pendapatan bulanan: Aktual vs Budget (Rp juta)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!B75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$B$76:$B$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!C75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="A3A19A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$C$76:$C$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="60"/>
+        <overlap val="-8"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBDB6"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E4E3DF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="t"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>EBITDA bulanan: Aktual vs Budget (Rp juta)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!D75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$D$76:$D$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!E75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="A3A19A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$E$76:$E$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="60"/>
+        <overlap val="-8"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBDB6"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E4E3DF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="t"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Produksi batubara bulanan (ton)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!F75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$F$76:$F$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!G75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="A3A19A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$G$76:$G$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="60"/>
+        <overlap val="-8"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBDB6"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E4E3DF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="t"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Stripping ratio (bcm/t): Aktual vs Budget</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!H75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="25400">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$H$76:$H$87</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!I75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="25400">
+              <a:solidFill>
+                <a:srgbClr val="A3A19A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="A3A19A"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$I$76:$I$87</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBDB6"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E4E3DF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="0.00" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="t"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cash cost FOB excl. royalti vs ASP (USD/t)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!J75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="25400">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$J$76:$J$87</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!K75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="25400">
+              <a:solidFill>
+                <a:srgbClr val="A3A19A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="A3A19A"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$K$76:$K$87</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!L75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="25400">
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$L$76:$L$87</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBDB6"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E4E3DF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="0.00" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="t"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Fuel ratio (L/bcm): Aktual vs Budget</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!M75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="25400">
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$M$76:$M$87</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!N75</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="25400">
+              <a:solidFill>
+                <a:srgbClr val="A3A19A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="A3A19A"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$76:$A$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$N$76:$N$87</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBDB6"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E4E3DF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="0.00" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="t"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Struktur biaya kas YTD (Rp juta)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!B90</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$91:$A$98</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$B$91:$B$98</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!C90</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="A3A19A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$91:$A$98</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$C$91:$C$98</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="60"/>
+        <overlap val="-8"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBDB6"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E4E3DF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="t"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Skor KPI per perspektif (skala 1–5)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!B101</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$A$102:$A$106</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$B$102:$B$106</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="60"/>
+        <overlap val="-8"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBDB6"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="5"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E4E3DF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="0.0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Jumlah KPI per status</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'C12 GEG Dashboard'!E101</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="0CA30C"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="0CA30C"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="FAB219"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="D03B3B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <cat>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$D$102:$D$104</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'C12 GEG Dashboard'!$E$102:$E$104</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBDB6"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E4E3DF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <spPr>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5940000" cy="2736000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5940000" cy="2736000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5940000" cy="2736000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5940000" cy="2736000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5940000" cy="2736000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5940000" cy="2736000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>57</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5940000" cy="2736000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="7" name="Chart 7"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>57</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5940000" cy="2736000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="8" name="Chart 8"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId8"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>18</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4320000" cy="2736000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="9" name="Chart 9"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -734,7 +2372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1040,83 +2678,83 @@
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>C12 GEG Dashboard</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>DASHBOARD: tile KPI, 8 grafik kinerja (pendapatan, EBITDA, produksi, SR, cash cost vs ASP, fuel ratio, struktur biaya, skor perspektif) + tabel KPI Scored</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>KODE WARNA</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n"/>
-      <c r="C30" s="5" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>1.234</t>
         </is>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>Teks biru / sel kuning muda = input (hardcode) – ganti dengan data Anda</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>1.234</t>
         </is>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Teks hitam = rumus</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>1.234</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Teks hijau = tautan antar-sheet</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>1.234</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>Sel kuning terang = parameter kunci / selector</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>CATATAN PENTING</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n"/>
-      <c r="C36" s="5" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="14" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="inlineStr">
-        <is>
-          <t>Bagian A &amp; B memakai perusahaan FIKTIF "PT Batubara Contoh Tbk" dengan format penyajian yang lazim di emiten batubara BEI. Angka ilustratif, BUKAN data emiten mana pun.</t>
-        </is>
-      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
@@ -1126,7 +2764,7 @@
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>Laporan keuangan asli emiten (PTBA, ITMG, AADI, BUMI, BYAN, dll.) dapat diunduh di www.idx.co.id untuk pembanding angka riil.</t>
+          <t>Bagian A &amp; B memakai perusahaan FIKTIF "PT Batubara Contoh Tbk" dengan format penyajian yang lazim di emiten batubara BEI. Angka ilustratif, BUKAN data emiten mana pun.</t>
         </is>
       </c>
     </row>
@@ -1138,7 +2776,7 @@
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>Bagian C terisi DATA CONTOH (Jan–Agu 2026) agar semua rumus terlihat bekerja. Ganti seluruh sel input dengan data GEG.</t>
+          <t>Laporan keuangan asli emiten (PTBA, ITMG, AADI, BUMI, BYAN, dll.) dapat diunduh di www.idx.co.id untuk pembanding angka riil.</t>
         </is>
       </c>
     </row>
@@ -1150,7 +2788,7 @@
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>Satuan uang: Rp juta. Harga &amp; tarif: USD. Volume: ton / bcm. Kurs dipakai untuk konversi per unit.</t>
+          <t>Bagian C terisi DATA CONTOH (Jan–Agu 2026) agar semua rumus terlihat bekerja. Ganti seluruh sel input dengan data GEG.</t>
         </is>
       </c>
     </row>
@@ -1161,6 +2799,18 @@
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>Satuan uang: Rp juta. Harga &amp; tarif: USD. Volume: ton / bcm. Kurs dipakai untuk konversi per unit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>Semua angka di laporan, COP dan KPI adalah rumus – bila input diubah, seluruh laporan ikut terhitung ulang.</t>
         </is>
@@ -1189,6 +2839,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -30252,6 +31903,2365 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:Y106"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.5" customWidth="1" min="1" max="1"/>
+    <col width="11.5" customWidth="1" min="2" max="2"/>
+    <col width="11.5" customWidth="1" min="3" max="3"/>
+    <col width="11.5" customWidth="1" min="4" max="4"/>
+    <col width="11.5" customWidth="1" min="5" max="5"/>
+    <col width="11.5" customWidth="1" min="6" max="6"/>
+    <col width="11.5" customWidth="1" min="7" max="7"/>
+    <col width="11.5" customWidth="1" min="8" max="8"/>
+    <col width="11.5" customWidth="1" min="9" max="9"/>
+    <col width="11.5" customWidth="1" min="10" max="10"/>
+    <col width="11.5" customWidth="1" min="11" max="11"/>
+    <col width="11.5" customWidth="1" min="12" max="12"/>
+    <col width="11.5" customWidth="1" min="13" max="13"/>
+    <col width="11.5" customWidth="1" min="14" max="14"/>
+    <col width="11.5" customWidth="1" min="15" max="15"/>
+    <col width="11.5" customWidth="1" min="16" max="16"/>
+    <col width="11.5" customWidth="1" min="17" max="17"/>
+    <col width="11.5" customWidth="1" min="18" max="18"/>
+    <col width="5" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="9" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="3" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GEG – Dashboard Kinerja &amp; KPI Scored</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <f>"PT Global Energy Group | Periode YTD Jan – "&amp;'C1 GEG Setting'!$C$7&amp;" "&amp;'C1 GEG Setting'!$C$5&amp;" | Ubah bulan laporan di sheet C1 – seluruh dashboard ikut berubah"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="93" t="inlineStr">
+        <is>
+          <t>PENDAPATAN YTD (Rp juta)</t>
+        </is>
+      </c>
+      <c r="D4" s="93" t="inlineStr">
+        <is>
+          <t>EBITDA YTD (Rp juta)</t>
+        </is>
+      </c>
+      <c r="G4" s="93" t="inlineStr">
+        <is>
+          <t>LABA BERSIH YTD (Rp juta)</t>
+        </is>
+      </c>
+      <c r="J4" s="93" t="inlineStr">
+        <is>
+          <t>PRODUKSI YTD (ton)</t>
+        </is>
+      </c>
+      <c r="M4" s="93" t="inlineStr">
+        <is>
+          <t>CASH COST FOB excl. royalti (USD/t)</t>
+        </is>
+      </c>
+      <c r="P4" s="93" t="inlineStr">
+        <is>
+          <t>SKOR KPI TERTIMBANG (1–5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="94">
+        <f>'C8 GEG Lap LR'!$J$13</f>
+        <v/>
+      </c>
+      <c r="D5" s="94">
+        <f>'C8 GEG Lap LR'!$J$85</f>
+        <v/>
+      </c>
+      <c r="G5" s="94">
+        <f>'C8 GEG Lap LR'!$J$82</f>
+        <v/>
+      </c>
+      <c r="J5" s="94">
+        <f>'C9 GEG Lap Ops'!$J$8</f>
+        <v/>
+      </c>
+      <c r="M5" s="95">
+        <f>'C10 GEG COP'!$L$19</f>
+        <v/>
+      </c>
+      <c r="P5" s="95">
+        <f>'C11 GEG KPI Scorecard'!$L$42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="96">
+        <f>"Budget: "&amp;TEXT('C8 GEG Lap LR'!$K$13,"#,##0")&amp;"  ("&amp;IF(IFERROR('C8 GEG Lap LR'!$J$13/'C8 GEG Lap LR'!$K$13-1,0)&gt;=0,"+","")&amp;TEXT(IFERROR('C8 GEG Lap LR'!$J$13/'C8 GEG Lap LR'!$K$13-1,0),"0.0%")&amp;")"</f>
+        <v/>
+      </c>
+      <c r="D6" s="96">
+        <f>"Budget: "&amp;TEXT('C8 GEG Lap LR'!$K$85,"#,##0")&amp;"  ("&amp;IF(IFERROR('C8 GEG Lap LR'!$J$85/'C8 GEG Lap LR'!$K$85-1,0)&gt;=0,"+","")&amp;TEXT(IFERROR('C8 GEG Lap LR'!$J$85/'C8 GEG Lap LR'!$K$85-1,0),"0.0%")&amp;")"</f>
+        <v/>
+      </c>
+      <c r="G6" s="96">
+        <f>"Budget: "&amp;TEXT('C8 GEG Lap LR'!$K$82,"#,##0")&amp;"  ("&amp;IF(IFERROR('C8 GEG Lap LR'!$J$82/'C8 GEG Lap LR'!$K$82-1,0)&gt;=0,"+","")&amp;TEXT(IFERROR('C8 GEG Lap LR'!$J$82/'C8 GEG Lap LR'!$K$82-1,0),"0.0%")&amp;")"</f>
+        <v/>
+      </c>
+      <c r="J6" s="96">
+        <f>"Budget: "&amp;TEXT('C9 GEG Lap Ops'!$K$8,"#,##0")&amp;"  ("&amp;IF(IFERROR('C9 GEG Lap Ops'!$J$8/'C9 GEG Lap Ops'!$K$8-1,0)&gt;=0,"+","")&amp;TEXT(IFERROR('C9 GEG Lap Ops'!$J$8/'C9 GEG Lap Ops'!$K$8-1,0),"0.0%")&amp;")"</f>
+        <v/>
+      </c>
+      <c r="M6" s="96">
+        <f>"Budget: "&amp;TEXT('C10 GEG COP'!$M$19,"#,##0.00")&amp;"  ("&amp;IF(IFERROR('C10 GEG COP'!$L$19/'C10 GEG COP'!$M$19-1,0)&gt;=0,"+","")&amp;TEXT(IFERROR('C10 GEG COP'!$L$19/'C10 GEG COP'!$M$19-1,0),"0.0%")&amp;")"</f>
+        <v/>
+      </c>
+      <c r="P6" s="97">
+        <f>"Predikat: "&amp;'C11 GEG KPI Scorecard'!$L$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="98">
+        <f>IF('C8 GEG Lap LR'!$J$13&gt;='C8 GEG Lap LR'!$K$13,"▲ Sesuai / lebih baik dari budget","▼ Lebih buruk dari budget")</f>
+        <v/>
+      </c>
+      <c r="D7" s="98">
+        <f>IF('C8 GEG Lap LR'!$J$85&gt;='C8 GEG Lap LR'!$K$85,"▲ Sesuai / lebih baik dari budget","▼ Lebih buruk dari budget")</f>
+        <v/>
+      </c>
+      <c r="G7" s="98">
+        <f>IF('C8 GEG Lap LR'!$J$82&gt;='C8 GEG Lap LR'!$K$82,"▲ Sesuai / lebih baik dari budget","▼ Lebih buruk dari budget")</f>
+        <v/>
+      </c>
+      <c r="J7" s="98">
+        <f>IF('C9 GEG Lap Ops'!$J$8&gt;='C9 GEG Lap Ops'!$K$8,"▲ Sesuai / lebih baik dari budget","▼ Lebih buruk dari budget")</f>
+        <v/>
+      </c>
+      <c r="M7" s="98">
+        <f>IF('C10 GEG COP'!$L$19&lt;='C10 GEG COP'!$M$19,"▲ Sesuai / lebih baik dari budget","▼ Lebih buruk dari budget")</f>
+        <v/>
+      </c>
+      <c r="P7" s="96">
+        <f>"Hijau "&amp;'C11 GEG KPI Scorecard'!$K$44&amp;" | Kuning "&amp;'C11 GEG KPI Scorecard'!$L$44&amp;" | Merah "&amp;'C11 GEG KPI Scorecard'!$M$44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>GRAFIK KINERJA BULANAN &amp; YTD</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
+      <c r="M9" s="5" t="n"/>
+      <c r="N9" s="5" t="n"/>
+      <c r="O9" s="5" t="n"/>
+      <c r="P9" s="5" t="n"/>
+      <c r="Q9" s="5" t="n"/>
+      <c r="R9" s="5" t="n"/>
+      <c r="S9" s="99" t="inlineStr">
+        <is>
+          <t>KPI SCORED – YTD</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="n"/>
+      <c r="U9" s="2" t="n"/>
+      <c r="V9" s="2" t="n"/>
+      <c r="W9" s="2" t="n"/>
+      <c r="X9" s="2" t="n"/>
+      <c r="Y9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="S10" s="100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T10" s="100" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="U10" s="100" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="V10" s="100" t="inlineStr">
+        <is>
+          <t>Aktual</t>
+        </is>
+      </c>
+      <c r="W10" s="100" t="inlineStr">
+        <is>
+          <t>Pencapaian</t>
+        </is>
+      </c>
+      <c r="X10" s="100" t="inlineStr">
+        <is>
+          <t>Skor</t>
+        </is>
+      </c>
+      <c r="Y10" s="100" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="S11" s="101">
+        <f>'C11 GEG KPI Scorecard'!$A$6</f>
+        <v/>
+      </c>
+      <c r="T11" s="5" t="n"/>
+      <c r="U11" s="5" t="n"/>
+      <c r="V11" s="5" t="n"/>
+      <c r="W11" s="5" t="n"/>
+      <c r="X11" s="5" t="n"/>
+      <c r="Y11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="S12" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$7</f>
+        <v/>
+      </c>
+      <c r="T12" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$7</f>
+        <v/>
+      </c>
+      <c r="U12" s="28">
+        <f>'C11 GEG KPI Scorecard'!$H$7</f>
+        <v/>
+      </c>
+      <c r="V12" s="28">
+        <f>'C11 GEG KPI Scorecard'!$I$7</f>
+        <v/>
+      </c>
+      <c r="W12" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$7</f>
+        <v/>
+      </c>
+      <c r="X12" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$7</f>
+        <v/>
+      </c>
+      <c r="Y12" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="S13" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$8</f>
+        <v/>
+      </c>
+      <c r="T13" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$8</f>
+        <v/>
+      </c>
+      <c r="U13" s="28">
+        <f>'C11 GEG KPI Scorecard'!$H$8</f>
+        <v/>
+      </c>
+      <c r="V13" s="28">
+        <f>'C11 GEG KPI Scorecard'!$I$8</f>
+        <v/>
+      </c>
+      <c r="W13" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$8</f>
+        <v/>
+      </c>
+      <c r="X13" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$8</f>
+        <v/>
+      </c>
+      <c r="Y13" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="S14" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$9</f>
+        <v/>
+      </c>
+      <c r="T14" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$9</f>
+        <v/>
+      </c>
+      <c r="U14" s="39">
+        <f>'C11 GEG KPI Scorecard'!$H$9</f>
+        <v/>
+      </c>
+      <c r="V14" s="39">
+        <f>'C11 GEG KPI Scorecard'!$I$9</f>
+        <v/>
+      </c>
+      <c r="W14" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$9</f>
+        <v/>
+      </c>
+      <c r="X14" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$9</f>
+        <v/>
+      </c>
+      <c r="Y14" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="S15" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$10</f>
+        <v/>
+      </c>
+      <c r="T15" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$10</f>
+        <v/>
+      </c>
+      <c r="U15" s="42">
+        <f>'C11 GEG KPI Scorecard'!$H$10</f>
+        <v/>
+      </c>
+      <c r="V15" s="42">
+        <f>'C11 GEG KPI Scorecard'!$I$10</f>
+        <v/>
+      </c>
+      <c r="W15" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$10</f>
+        <v/>
+      </c>
+      <c r="X15" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$10</f>
+        <v/>
+      </c>
+      <c r="Y15" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="S16" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$11</f>
+        <v/>
+      </c>
+      <c r="T16" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$11</f>
+        <v/>
+      </c>
+      <c r="U16" s="90">
+        <f>'C11 GEG KPI Scorecard'!$H$11</f>
+        <v/>
+      </c>
+      <c r="V16" s="90">
+        <f>'C11 GEG KPI Scorecard'!$I$11</f>
+        <v/>
+      </c>
+      <c r="W16" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$11</f>
+        <v/>
+      </c>
+      <c r="X16" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$11</f>
+        <v/>
+      </c>
+      <c r="Y16" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="S17" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$12</f>
+        <v/>
+      </c>
+      <c r="T17" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$12</f>
+        <v/>
+      </c>
+      <c r="U17" s="42">
+        <f>'C11 GEG KPI Scorecard'!$H$12</f>
+        <v/>
+      </c>
+      <c r="V17" s="42">
+        <f>'C11 GEG KPI Scorecard'!$I$12</f>
+        <v/>
+      </c>
+      <c r="W17" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$12</f>
+        <v/>
+      </c>
+      <c r="X17" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$12</f>
+        <v/>
+      </c>
+      <c r="Y17" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="S18" s="101">
+        <f>'C11 GEG KPI Scorecard'!$A$13</f>
+        <v/>
+      </c>
+      <c r="T18" s="5" t="n"/>
+      <c r="U18" s="5" t="n"/>
+      <c r="V18" s="5" t="n"/>
+      <c r="W18" s="5" t="n"/>
+      <c r="X18" s="5" t="n"/>
+      <c r="Y18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="S19" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$14</f>
+        <v/>
+      </c>
+      <c r="T19" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$14</f>
+        <v/>
+      </c>
+      <c r="U19" s="39">
+        <f>'C11 GEG KPI Scorecard'!$H$14</f>
+        <v/>
+      </c>
+      <c r="V19" s="39">
+        <f>'C11 GEG KPI Scorecard'!$I$14</f>
+        <v/>
+      </c>
+      <c r="W19" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$14</f>
+        <v/>
+      </c>
+      <c r="X19" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$14</f>
+        <v/>
+      </c>
+      <c r="Y19" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="S20" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$15</f>
+        <v/>
+      </c>
+      <c r="T20" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$15</f>
+        <v/>
+      </c>
+      <c r="U20" s="39">
+        <f>'C11 GEG KPI Scorecard'!$H$15</f>
+        <v/>
+      </c>
+      <c r="V20" s="39">
+        <f>'C11 GEG KPI Scorecard'!$I$15</f>
+        <v/>
+      </c>
+      <c r="W20" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$15</f>
+        <v/>
+      </c>
+      <c r="X20" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$15</f>
+        <v/>
+      </c>
+      <c r="Y20" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="S21" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$16</f>
+        <v/>
+      </c>
+      <c r="T21" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$16</f>
+        <v/>
+      </c>
+      <c r="U21" s="39">
+        <f>'C11 GEG KPI Scorecard'!$H$16</f>
+        <v/>
+      </c>
+      <c r="V21" s="39">
+        <f>'C11 GEG KPI Scorecard'!$I$16</f>
+        <v/>
+      </c>
+      <c r="W21" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$16</f>
+        <v/>
+      </c>
+      <c r="X21" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$16</f>
+        <v/>
+      </c>
+      <c r="Y21" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="S22" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$17</f>
+        <v/>
+      </c>
+      <c r="T22" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$17</f>
+        <v/>
+      </c>
+      <c r="U22" s="56">
+        <f>'C11 GEG KPI Scorecard'!$H$17</f>
+        <v/>
+      </c>
+      <c r="V22" s="56">
+        <f>'C11 GEG KPI Scorecard'!$I$17</f>
+        <v/>
+      </c>
+      <c r="W22" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$17</f>
+        <v/>
+      </c>
+      <c r="X22" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$17</f>
+        <v/>
+      </c>
+      <c r="Y22" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="S23" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$18</f>
+        <v/>
+      </c>
+      <c r="T23" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$18</f>
+        <v/>
+      </c>
+      <c r="U23" s="39">
+        <f>'C11 GEG KPI Scorecard'!$H$18</f>
+        <v/>
+      </c>
+      <c r="V23" s="39">
+        <f>'C11 GEG KPI Scorecard'!$I$18</f>
+        <v/>
+      </c>
+      <c r="W23" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$18</f>
+        <v/>
+      </c>
+      <c r="X23" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$18</f>
+        <v/>
+      </c>
+      <c r="Y23" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="S24" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$19</f>
+        <v/>
+      </c>
+      <c r="T24" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$19</f>
+        <v/>
+      </c>
+      <c r="U24" s="39">
+        <f>'C11 GEG KPI Scorecard'!$H$19</f>
+        <v/>
+      </c>
+      <c r="V24" s="39">
+        <f>'C11 GEG KPI Scorecard'!$I$19</f>
+        <v/>
+      </c>
+      <c r="W24" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$19</f>
+        <v/>
+      </c>
+      <c r="X24" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$19</f>
+        <v/>
+      </c>
+      <c r="Y24" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="S25" s="101">
+        <f>'C11 GEG KPI Scorecard'!$A$20</f>
+        <v/>
+      </c>
+      <c r="T25" s="5" t="n"/>
+      <c r="U25" s="5" t="n"/>
+      <c r="V25" s="5" t="n"/>
+      <c r="W25" s="5" t="n"/>
+      <c r="X25" s="5" t="n"/>
+      <c r="Y25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="S26" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$21</f>
+        <v/>
+      </c>
+      <c r="T26" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$21</f>
+        <v/>
+      </c>
+      <c r="U26" s="42">
+        <f>'C11 GEG KPI Scorecard'!$H$21</f>
+        <v/>
+      </c>
+      <c r="V26" s="42">
+        <f>'C11 GEG KPI Scorecard'!$I$21</f>
+        <v/>
+      </c>
+      <c r="W26" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$21</f>
+        <v/>
+      </c>
+      <c r="X26" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$21</f>
+        <v/>
+      </c>
+      <c r="Y26" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="S27" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$22</f>
+        <v/>
+      </c>
+      <c r="T27" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$22</f>
+        <v/>
+      </c>
+      <c r="U27" s="28">
+        <f>'C11 GEG KPI Scorecard'!$H$22</f>
+        <v/>
+      </c>
+      <c r="V27" s="28">
+        <f>'C11 GEG KPI Scorecard'!$I$22</f>
+        <v/>
+      </c>
+      <c r="W27" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$22</f>
+        <v/>
+      </c>
+      <c r="X27" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$22</f>
+        <v/>
+      </c>
+      <c r="Y27" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="S28" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$23</f>
+        <v/>
+      </c>
+      <c r="T28" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$23</f>
+        <v/>
+      </c>
+      <c r="U28" s="42">
+        <f>'C11 GEG KPI Scorecard'!$H$23</f>
+        <v/>
+      </c>
+      <c r="V28" s="42">
+        <f>'C11 GEG KPI Scorecard'!$I$23</f>
+        <v/>
+      </c>
+      <c r="W28" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$23</f>
+        <v/>
+      </c>
+      <c r="X28" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$23</f>
+        <v/>
+      </c>
+      <c r="Y28" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="S29" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$24</f>
+        <v/>
+      </c>
+      <c r="T29" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$24</f>
+        <v/>
+      </c>
+      <c r="U29" s="39">
+        <f>'C11 GEG KPI Scorecard'!$H$24</f>
+        <v/>
+      </c>
+      <c r="V29" s="39">
+        <f>'C11 GEG KPI Scorecard'!$I$24</f>
+        <v/>
+      </c>
+      <c r="W29" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$24</f>
+        <v/>
+      </c>
+      <c r="X29" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$24</f>
+        <v/>
+      </c>
+      <c r="Y29" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="S30" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$25</f>
+        <v/>
+      </c>
+      <c r="T30" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$25</f>
+        <v/>
+      </c>
+      <c r="U30" s="28">
+        <f>'C11 GEG KPI Scorecard'!$H$25</f>
+        <v/>
+      </c>
+      <c r="V30" s="28">
+        <f>'C11 GEG KPI Scorecard'!$I$25</f>
+        <v/>
+      </c>
+      <c r="W30" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$25</f>
+        <v/>
+      </c>
+      <c r="X30" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$25</f>
+        <v/>
+      </c>
+      <c r="Y30" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="S31" s="101">
+        <f>'C11 GEG KPI Scorecard'!$A$26</f>
+        <v/>
+      </c>
+      <c r="T31" s="5" t="n"/>
+      <c r="U31" s="5" t="n"/>
+      <c r="V31" s="5" t="n"/>
+      <c r="W31" s="5" t="n"/>
+      <c r="X31" s="5" t="n"/>
+      <c r="Y31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="S32" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$27</f>
+        <v/>
+      </c>
+      <c r="T32" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$27</f>
+        <v/>
+      </c>
+      <c r="U32" s="28">
+        <f>'C11 GEG KPI Scorecard'!$H$27</f>
+        <v/>
+      </c>
+      <c r="V32" s="28">
+        <f>'C11 GEG KPI Scorecard'!$I$27</f>
+        <v/>
+      </c>
+      <c r="W32" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$27</f>
+        <v/>
+      </c>
+      <c r="X32" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$27</f>
+        <v/>
+      </c>
+      <c r="Y32" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="S33" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$28</f>
+        <v/>
+      </c>
+      <c r="T33" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$28</f>
+        <v/>
+      </c>
+      <c r="U33" s="28">
+        <f>'C11 GEG KPI Scorecard'!$H$28</f>
+        <v/>
+      </c>
+      <c r="V33" s="28">
+        <f>'C11 GEG KPI Scorecard'!$I$28</f>
+        <v/>
+      </c>
+      <c r="W33" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$28</f>
+        <v/>
+      </c>
+      <c r="X33" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$28</f>
+        <v/>
+      </c>
+      <c r="Y33" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="S34" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$29</f>
+        <v/>
+      </c>
+      <c r="T34" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$29</f>
+        <v/>
+      </c>
+      <c r="U34" s="42">
+        <f>'C11 GEG KPI Scorecard'!$H$29</f>
+        <v/>
+      </c>
+      <c r="V34" s="42">
+        <f>'C11 GEG KPI Scorecard'!$I$29</f>
+        <v/>
+      </c>
+      <c r="W34" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$29</f>
+        <v/>
+      </c>
+      <c r="X34" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$29</f>
+        <v/>
+      </c>
+      <c r="Y34" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="S35" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$30</f>
+        <v/>
+      </c>
+      <c r="T35" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$30</f>
+        <v/>
+      </c>
+      <c r="U35" s="42">
+        <f>'C11 GEG KPI Scorecard'!$H$30</f>
+        <v/>
+      </c>
+      <c r="V35" s="42">
+        <f>'C11 GEG KPI Scorecard'!$I$30</f>
+        <v/>
+      </c>
+      <c r="W35" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$30</f>
+        <v/>
+      </c>
+      <c r="X35" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$30</f>
+        <v/>
+      </c>
+      <c r="Y35" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="S36" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$31</f>
+        <v/>
+      </c>
+      <c r="T36" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$31</f>
+        <v/>
+      </c>
+      <c r="U36" s="28">
+        <f>'C11 GEG KPI Scorecard'!$H$31</f>
+        <v/>
+      </c>
+      <c r="V36" s="28">
+        <f>'C11 GEG KPI Scorecard'!$I$31</f>
+        <v/>
+      </c>
+      <c r="W36" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$31</f>
+        <v/>
+      </c>
+      <c r="X36" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$31</f>
+        <v/>
+      </c>
+      <c r="Y36" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="S37" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$32</f>
+        <v/>
+      </c>
+      <c r="T37" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$32</f>
+        <v/>
+      </c>
+      <c r="U37" s="42">
+        <f>'C11 GEG KPI Scorecard'!$H$32</f>
+        <v/>
+      </c>
+      <c r="V37" s="42">
+        <f>'C11 GEG KPI Scorecard'!$I$32</f>
+        <v/>
+      </c>
+      <c r="W37" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$32</f>
+        <v/>
+      </c>
+      <c r="X37" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$32</f>
+        <v/>
+      </c>
+      <c r="Y37" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="S38" s="101">
+        <f>'C11 GEG KPI Scorecard'!$A$33</f>
+        <v/>
+      </c>
+      <c r="T38" s="5" t="n"/>
+      <c r="U38" s="5" t="n"/>
+      <c r="V38" s="5" t="n"/>
+      <c r="W38" s="5" t="n"/>
+      <c r="X38" s="5" t="n"/>
+      <c r="Y38" s="5" t="n"/>
+    </row>
+    <row r="39">
+      <c r="S39" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$34</f>
+        <v/>
+      </c>
+      <c r="T39" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$34</f>
+        <v/>
+      </c>
+      <c r="U39" s="88">
+        <f>'C11 GEG KPI Scorecard'!$H$34</f>
+        <v/>
+      </c>
+      <c r="V39" s="88">
+        <f>'C11 GEG KPI Scorecard'!$I$34</f>
+        <v/>
+      </c>
+      <c r="W39" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$34</f>
+        <v/>
+      </c>
+      <c r="X39" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$34</f>
+        <v/>
+      </c>
+      <c r="Y39" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="S40" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$35</f>
+        <v/>
+      </c>
+      <c r="T40" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$35</f>
+        <v/>
+      </c>
+      <c r="U40" s="64">
+        <f>'C11 GEG KPI Scorecard'!$H$35</f>
+        <v/>
+      </c>
+      <c r="V40" s="64">
+        <f>'C11 GEG KPI Scorecard'!$I$35</f>
+        <v/>
+      </c>
+      <c r="W40" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$35</f>
+        <v/>
+      </c>
+      <c r="X40" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$35</f>
+        <v/>
+      </c>
+      <c r="Y40" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="S41" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$36</f>
+        <v/>
+      </c>
+      <c r="T41" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$36</f>
+        <v/>
+      </c>
+      <c r="U41" s="64">
+        <f>'C11 GEG KPI Scorecard'!$H$36</f>
+        <v/>
+      </c>
+      <c r="V41" s="64">
+        <f>'C11 GEG KPI Scorecard'!$I$36</f>
+        <v/>
+      </c>
+      <c r="W41" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$36</f>
+        <v/>
+      </c>
+      <c r="X41" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$36</f>
+        <v/>
+      </c>
+      <c r="Y41" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="S42" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$37</f>
+        <v/>
+      </c>
+      <c r="T42" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$37</f>
+        <v/>
+      </c>
+      <c r="U42" s="39">
+        <f>'C11 GEG KPI Scorecard'!$H$37</f>
+        <v/>
+      </c>
+      <c r="V42" s="39">
+        <f>'C11 GEG KPI Scorecard'!$I$37</f>
+        <v/>
+      </c>
+      <c r="W42" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$37</f>
+        <v/>
+      </c>
+      <c r="X42" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$37</f>
+        <v/>
+      </c>
+      <c r="Y42" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="S43" s="59">
+        <f>'C11 GEG KPI Scorecard'!$A$38</f>
+        <v/>
+      </c>
+      <c r="T43" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$38</f>
+        <v/>
+      </c>
+      <c r="U43" s="88">
+        <f>'C11 GEG KPI Scorecard'!$H$38</f>
+        <v/>
+      </c>
+      <c r="V43" s="88">
+        <f>'C11 GEG KPI Scorecard'!$I$38</f>
+        <v/>
+      </c>
+      <c r="W43" s="42">
+        <f>'C11 GEG KPI Scorecard'!$J$38</f>
+        <v/>
+      </c>
+      <c r="X43" s="59">
+        <f>'C11 GEG KPI Scorecard'!$K$38</f>
+        <v/>
+      </c>
+      <c r="Y43" s="12">
+        <f>'C11 GEG KPI Scorecard'!$M$38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="T44" s="46" t="inlineStr">
+        <is>
+          <t>SKOR TERTIMBANG TOTAL</t>
+        </is>
+      </c>
+      <c r="X44" s="103">
+        <f>'C11 GEG KPI Scorecard'!$L$42</f>
+        <v/>
+      </c>
+      <c r="Y44" s="104">
+        <f>'C11 GEG KPI Scorecard'!$L$43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="T45" s="3" t="inlineStr">
+        <is>
+          <t>Skor 1–5 per KPI; status Hijau ≥100%, Kuning ≥95%, Merah &lt;95% dari target (atur di C1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>DATA GRAFIK (otomatis – jangan diubah). #N/A = bulan setelah bulan laporan, sengaja agar grafik tidak jatuh ke nol.</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="n"/>
+      <c r="C74" s="5" t="n"/>
+      <c r="D74" s="5" t="n"/>
+      <c r="E74" s="5" t="n"/>
+      <c r="F74" s="5" t="n"/>
+      <c r="G74" s="5" t="n"/>
+      <c r="H74" s="5" t="n"/>
+      <c r="I74" s="5" t="n"/>
+      <c r="J74" s="5" t="n"/>
+      <c r="K74" s="5" t="n"/>
+      <c r="L74" s="5" t="n"/>
+      <c r="M74" s="5" t="n"/>
+      <c r="N74" s="5" t="n"/>
+      <c r="O74" s="5" t="n"/>
+      <c r="P74" s="5" t="n"/>
+      <c r="Q74" s="5" t="n"/>
+      <c r="R74" s="5" t="n"/>
+    </row>
+    <row r="75" ht="42" customHeight="1">
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t>Bulan</t>
+        </is>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>Pendapatan Aktual</t>
+        </is>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>Pendapatan Budget</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>EBITDA Aktual</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>EBITDA Budget</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>Produksi Aktual (t)</t>
+        </is>
+      </c>
+      <c r="G75" s="16" t="inlineStr">
+        <is>
+          <t>Produksi Budget (t)</t>
+        </is>
+      </c>
+      <c r="H75" s="16" t="inlineStr">
+        <is>
+          <t>SR Aktual</t>
+        </is>
+      </c>
+      <c r="I75" s="16" t="inlineStr">
+        <is>
+          <t>SR Budget</t>
+        </is>
+      </c>
+      <c r="J75" s="16" t="inlineStr">
+        <is>
+          <t>Cash cost Aktual (USD/t)</t>
+        </is>
+      </c>
+      <c r="K75" s="16" t="inlineStr">
+        <is>
+          <t>Cash cost Budget (USD/t)</t>
+        </is>
+      </c>
+      <c r="L75" s="16" t="inlineStr">
+        <is>
+          <t>ASP Aktual (USD/t)</t>
+        </is>
+      </c>
+      <c r="M75" s="16" t="inlineStr">
+        <is>
+          <t>Fuel ratio Aktual</t>
+        </is>
+      </c>
+      <c r="N75" s="16" t="inlineStr">
+        <is>
+          <t>Fuel ratio Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B76" s="28">
+        <f>IF(1&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!D14)</f>
+        <v/>
+      </c>
+      <c r="C76" s="28">
+        <f>'C4 GEG LR Budget'!D14</f>
+        <v/>
+      </c>
+      <c r="D76" s="28">
+        <f>IF(1&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!D86)</f>
+        <v/>
+      </c>
+      <c r="E76" s="28">
+        <f>'C4 GEG LR Budget'!D86</f>
+        <v/>
+      </c>
+      <c r="F76" s="28">
+        <f>IF(1&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!D9)</f>
+        <v/>
+      </c>
+      <c r="G76" s="28">
+        <f>'C2 GEG Ops Budget'!D9</f>
+        <v/>
+      </c>
+      <c r="H76" s="39">
+        <f>IF(1&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!D10)</f>
+        <v/>
+      </c>
+      <c r="I76" s="39">
+        <f>'C2 GEG Ops Budget'!D10</f>
+        <v/>
+      </c>
+      <c r="J76" s="39">
+        <f>IF(1&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!D25+'C5 GEG LR Aktual'!D31+'C5 GEG LR Aktual'!D41)*1000000/'C3 GEG Ops Aktual'!D19/'C3 GEG Ops Aktual'!D25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K76" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!D25+'C4 GEG LR Budget'!D31+'C4 GEG LR Budget'!D41)*1000000/'C2 GEG Ops Budget'!D19/'C2 GEG Ops Budget'!D25,NA())</f>
+        <v/>
+      </c>
+      <c r="L76" s="39">
+        <f>IF(1&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!D11+'C5 GEG LR Aktual'!D12)*1000000/'C3 GEG Ops Aktual'!D19/'C3 GEG Ops Aktual'!D25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M76" s="39">
+        <f>IF(1&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!D28)</f>
+        <v/>
+      </c>
+      <c r="N76" s="39">
+        <f>'C2 GEG Ops Budget'!D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B77" s="28">
+        <f>IF(2&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!E14)</f>
+        <v/>
+      </c>
+      <c r="C77" s="28">
+        <f>'C4 GEG LR Budget'!E14</f>
+        <v/>
+      </c>
+      <c r="D77" s="28">
+        <f>IF(2&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!E86)</f>
+        <v/>
+      </c>
+      <c r="E77" s="28">
+        <f>'C4 GEG LR Budget'!E86</f>
+        <v/>
+      </c>
+      <c r="F77" s="28">
+        <f>IF(2&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!E9)</f>
+        <v/>
+      </c>
+      <c r="G77" s="28">
+        <f>'C2 GEG Ops Budget'!E9</f>
+        <v/>
+      </c>
+      <c r="H77" s="39">
+        <f>IF(2&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!E10)</f>
+        <v/>
+      </c>
+      <c r="I77" s="39">
+        <f>'C2 GEG Ops Budget'!E10</f>
+        <v/>
+      </c>
+      <c r="J77" s="39">
+        <f>IF(2&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!E25+'C5 GEG LR Aktual'!E31+'C5 GEG LR Aktual'!E41)*1000000/'C3 GEG Ops Aktual'!E19/'C3 GEG Ops Aktual'!E25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K77" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!E25+'C4 GEG LR Budget'!E31+'C4 GEG LR Budget'!E41)*1000000/'C2 GEG Ops Budget'!E19/'C2 GEG Ops Budget'!E25,NA())</f>
+        <v/>
+      </c>
+      <c r="L77" s="39">
+        <f>IF(2&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!E11+'C5 GEG LR Aktual'!E12)*1000000/'C3 GEG Ops Aktual'!E19/'C3 GEG Ops Aktual'!E25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M77" s="39">
+        <f>IF(2&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!E28)</f>
+        <v/>
+      </c>
+      <c r="N77" s="39">
+        <f>'C2 GEG Ops Budget'!E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B78" s="28">
+        <f>IF(3&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!F14)</f>
+        <v/>
+      </c>
+      <c r="C78" s="28">
+        <f>'C4 GEG LR Budget'!F14</f>
+        <v/>
+      </c>
+      <c r="D78" s="28">
+        <f>IF(3&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!F86)</f>
+        <v/>
+      </c>
+      <c r="E78" s="28">
+        <f>'C4 GEG LR Budget'!F86</f>
+        <v/>
+      </c>
+      <c r="F78" s="28">
+        <f>IF(3&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!F9)</f>
+        <v/>
+      </c>
+      <c r="G78" s="28">
+        <f>'C2 GEG Ops Budget'!F9</f>
+        <v/>
+      </c>
+      <c r="H78" s="39">
+        <f>IF(3&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!F10)</f>
+        <v/>
+      </c>
+      <c r="I78" s="39">
+        <f>'C2 GEG Ops Budget'!F10</f>
+        <v/>
+      </c>
+      <c r="J78" s="39">
+        <f>IF(3&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!F25+'C5 GEG LR Aktual'!F31+'C5 GEG LR Aktual'!F41)*1000000/'C3 GEG Ops Aktual'!F19/'C3 GEG Ops Aktual'!F25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K78" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!F25+'C4 GEG LR Budget'!F31+'C4 GEG LR Budget'!F41)*1000000/'C2 GEG Ops Budget'!F19/'C2 GEG Ops Budget'!F25,NA())</f>
+        <v/>
+      </c>
+      <c r="L78" s="39">
+        <f>IF(3&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!F11+'C5 GEG LR Aktual'!F12)*1000000/'C3 GEG Ops Aktual'!F19/'C3 GEG Ops Aktual'!F25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M78" s="39">
+        <f>IF(3&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!F28)</f>
+        <v/>
+      </c>
+      <c r="N78" s="39">
+        <f>'C2 GEG Ops Budget'!F28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="B79" s="28">
+        <f>IF(4&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!G14)</f>
+        <v/>
+      </c>
+      <c r="C79" s="28">
+        <f>'C4 GEG LR Budget'!G14</f>
+        <v/>
+      </c>
+      <c r="D79" s="28">
+        <f>IF(4&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!G86)</f>
+        <v/>
+      </c>
+      <c r="E79" s="28">
+        <f>'C4 GEG LR Budget'!G86</f>
+        <v/>
+      </c>
+      <c r="F79" s="28">
+        <f>IF(4&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!G9)</f>
+        <v/>
+      </c>
+      <c r="G79" s="28">
+        <f>'C2 GEG Ops Budget'!G9</f>
+        <v/>
+      </c>
+      <c r="H79" s="39">
+        <f>IF(4&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!G10)</f>
+        <v/>
+      </c>
+      <c r="I79" s="39">
+        <f>'C2 GEG Ops Budget'!G10</f>
+        <v/>
+      </c>
+      <c r="J79" s="39">
+        <f>IF(4&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!G25+'C5 GEG LR Aktual'!G31+'C5 GEG LR Aktual'!G41)*1000000/'C3 GEG Ops Aktual'!G19/'C3 GEG Ops Aktual'!G25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K79" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!G25+'C4 GEG LR Budget'!G31+'C4 GEG LR Budget'!G41)*1000000/'C2 GEG Ops Budget'!G19/'C2 GEG Ops Budget'!G25,NA())</f>
+        <v/>
+      </c>
+      <c r="L79" s="39">
+        <f>IF(4&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!G11+'C5 GEG LR Aktual'!G12)*1000000/'C3 GEG Ops Aktual'!G19/'C3 GEG Ops Aktual'!G25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M79" s="39">
+        <f>IF(4&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!G28)</f>
+        <v/>
+      </c>
+      <c r="N79" s="39">
+        <f>'C2 GEG Ops Budget'!G28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>Mei</t>
+        </is>
+      </c>
+      <c r="B80" s="28">
+        <f>IF(5&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!H14)</f>
+        <v/>
+      </c>
+      <c r="C80" s="28">
+        <f>'C4 GEG LR Budget'!H14</f>
+        <v/>
+      </c>
+      <c r="D80" s="28">
+        <f>IF(5&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!H86)</f>
+        <v/>
+      </c>
+      <c r="E80" s="28">
+        <f>'C4 GEG LR Budget'!H86</f>
+        <v/>
+      </c>
+      <c r="F80" s="28">
+        <f>IF(5&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!H9)</f>
+        <v/>
+      </c>
+      <c r="G80" s="28">
+        <f>'C2 GEG Ops Budget'!H9</f>
+        <v/>
+      </c>
+      <c r="H80" s="39">
+        <f>IF(5&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!H10)</f>
+        <v/>
+      </c>
+      <c r="I80" s="39">
+        <f>'C2 GEG Ops Budget'!H10</f>
+        <v/>
+      </c>
+      <c r="J80" s="39">
+        <f>IF(5&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!H25+'C5 GEG LR Aktual'!H31+'C5 GEG LR Aktual'!H41)*1000000/'C3 GEG Ops Aktual'!H19/'C3 GEG Ops Aktual'!H25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K80" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!H25+'C4 GEG LR Budget'!H31+'C4 GEG LR Budget'!H41)*1000000/'C2 GEG Ops Budget'!H19/'C2 GEG Ops Budget'!H25,NA())</f>
+        <v/>
+      </c>
+      <c r="L80" s="39">
+        <f>IF(5&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!H11+'C5 GEG LR Aktual'!H12)*1000000/'C3 GEG Ops Aktual'!H19/'C3 GEG Ops Aktual'!H25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M80" s="39">
+        <f>IF(5&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!H28)</f>
+        <v/>
+      </c>
+      <c r="N80" s="39">
+        <f>'C2 GEG Ops Budget'!H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="B81" s="28">
+        <f>IF(6&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!I14)</f>
+        <v/>
+      </c>
+      <c r="C81" s="28">
+        <f>'C4 GEG LR Budget'!I14</f>
+        <v/>
+      </c>
+      <c r="D81" s="28">
+        <f>IF(6&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!I86)</f>
+        <v/>
+      </c>
+      <c r="E81" s="28">
+        <f>'C4 GEG LR Budget'!I86</f>
+        <v/>
+      </c>
+      <c r="F81" s="28">
+        <f>IF(6&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!I9)</f>
+        <v/>
+      </c>
+      <c r="G81" s="28">
+        <f>'C2 GEG Ops Budget'!I9</f>
+        <v/>
+      </c>
+      <c r="H81" s="39">
+        <f>IF(6&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!I10)</f>
+        <v/>
+      </c>
+      <c r="I81" s="39">
+        <f>'C2 GEG Ops Budget'!I10</f>
+        <v/>
+      </c>
+      <c r="J81" s="39">
+        <f>IF(6&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!I25+'C5 GEG LR Aktual'!I31+'C5 GEG LR Aktual'!I41)*1000000/'C3 GEG Ops Aktual'!I19/'C3 GEG Ops Aktual'!I25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K81" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!I25+'C4 GEG LR Budget'!I31+'C4 GEG LR Budget'!I41)*1000000/'C2 GEG Ops Budget'!I19/'C2 GEG Ops Budget'!I25,NA())</f>
+        <v/>
+      </c>
+      <c r="L81" s="39">
+        <f>IF(6&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!I11+'C5 GEG LR Aktual'!I12)*1000000/'C3 GEG Ops Aktual'!I19/'C3 GEG Ops Aktual'!I25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M81" s="39">
+        <f>IF(6&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!I28)</f>
+        <v/>
+      </c>
+      <c r="N81" s="39">
+        <f>'C2 GEG Ops Budget'!I28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="B82" s="28">
+        <f>IF(7&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!J14)</f>
+        <v/>
+      </c>
+      <c r="C82" s="28">
+        <f>'C4 GEG LR Budget'!J14</f>
+        <v/>
+      </c>
+      <c r="D82" s="28">
+        <f>IF(7&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!J86)</f>
+        <v/>
+      </c>
+      <c r="E82" s="28">
+        <f>'C4 GEG LR Budget'!J86</f>
+        <v/>
+      </c>
+      <c r="F82" s="28">
+        <f>IF(7&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!J9)</f>
+        <v/>
+      </c>
+      <c r="G82" s="28">
+        <f>'C2 GEG Ops Budget'!J9</f>
+        <v/>
+      </c>
+      <c r="H82" s="39">
+        <f>IF(7&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!J10)</f>
+        <v/>
+      </c>
+      <c r="I82" s="39">
+        <f>'C2 GEG Ops Budget'!J10</f>
+        <v/>
+      </c>
+      <c r="J82" s="39">
+        <f>IF(7&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!J25+'C5 GEG LR Aktual'!J31+'C5 GEG LR Aktual'!J41)*1000000/'C3 GEG Ops Aktual'!J19/'C3 GEG Ops Aktual'!J25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K82" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!J25+'C4 GEG LR Budget'!J31+'C4 GEG LR Budget'!J41)*1000000/'C2 GEG Ops Budget'!J19/'C2 GEG Ops Budget'!J25,NA())</f>
+        <v/>
+      </c>
+      <c r="L82" s="39">
+        <f>IF(7&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!J11+'C5 GEG LR Aktual'!J12)*1000000/'C3 GEG Ops Aktual'!J19/'C3 GEG Ops Aktual'!J25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M82" s="39">
+        <f>IF(7&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!J28)</f>
+        <v/>
+      </c>
+      <c r="N82" s="39">
+        <f>'C2 GEG Ops Budget'!J28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>Agu</t>
+        </is>
+      </c>
+      <c r="B83" s="28">
+        <f>IF(8&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!K14)</f>
+        <v/>
+      </c>
+      <c r="C83" s="28">
+        <f>'C4 GEG LR Budget'!K14</f>
+        <v/>
+      </c>
+      <c r="D83" s="28">
+        <f>IF(8&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!K86)</f>
+        <v/>
+      </c>
+      <c r="E83" s="28">
+        <f>'C4 GEG LR Budget'!K86</f>
+        <v/>
+      </c>
+      <c r="F83" s="28">
+        <f>IF(8&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!K9)</f>
+        <v/>
+      </c>
+      <c r="G83" s="28">
+        <f>'C2 GEG Ops Budget'!K9</f>
+        <v/>
+      </c>
+      <c r="H83" s="39">
+        <f>IF(8&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!K10)</f>
+        <v/>
+      </c>
+      <c r="I83" s="39">
+        <f>'C2 GEG Ops Budget'!K10</f>
+        <v/>
+      </c>
+      <c r="J83" s="39">
+        <f>IF(8&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!K25+'C5 GEG LR Aktual'!K31+'C5 GEG LR Aktual'!K41)*1000000/'C3 GEG Ops Aktual'!K19/'C3 GEG Ops Aktual'!K25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K83" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!K25+'C4 GEG LR Budget'!K31+'C4 GEG LR Budget'!K41)*1000000/'C2 GEG Ops Budget'!K19/'C2 GEG Ops Budget'!K25,NA())</f>
+        <v/>
+      </c>
+      <c r="L83" s="39">
+        <f>IF(8&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!K11+'C5 GEG LR Aktual'!K12)*1000000/'C3 GEG Ops Aktual'!K19/'C3 GEG Ops Aktual'!K25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M83" s="39">
+        <f>IF(8&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!K28)</f>
+        <v/>
+      </c>
+      <c r="N83" s="39">
+        <f>'C2 GEG Ops Budget'!K28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="B84" s="28">
+        <f>IF(9&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!L14)</f>
+        <v/>
+      </c>
+      <c r="C84" s="28">
+        <f>'C4 GEG LR Budget'!L14</f>
+        <v/>
+      </c>
+      <c r="D84" s="28">
+        <f>IF(9&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!L86)</f>
+        <v/>
+      </c>
+      <c r="E84" s="28">
+        <f>'C4 GEG LR Budget'!L86</f>
+        <v/>
+      </c>
+      <c r="F84" s="28">
+        <f>IF(9&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!L9)</f>
+        <v/>
+      </c>
+      <c r="G84" s="28">
+        <f>'C2 GEG Ops Budget'!L9</f>
+        <v/>
+      </c>
+      <c r="H84" s="39">
+        <f>IF(9&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!L10)</f>
+        <v/>
+      </c>
+      <c r="I84" s="39">
+        <f>'C2 GEG Ops Budget'!L10</f>
+        <v/>
+      </c>
+      <c r="J84" s="39">
+        <f>IF(9&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!L25+'C5 GEG LR Aktual'!L31+'C5 GEG LR Aktual'!L41)*1000000/'C3 GEG Ops Aktual'!L19/'C3 GEG Ops Aktual'!L25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K84" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!L25+'C4 GEG LR Budget'!L31+'C4 GEG LR Budget'!L41)*1000000/'C2 GEG Ops Budget'!L19/'C2 GEG Ops Budget'!L25,NA())</f>
+        <v/>
+      </c>
+      <c r="L84" s="39">
+        <f>IF(9&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!L11+'C5 GEG LR Aktual'!L12)*1000000/'C3 GEG Ops Aktual'!L19/'C3 GEG Ops Aktual'!L25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M84" s="39">
+        <f>IF(9&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!L28)</f>
+        <v/>
+      </c>
+      <c r="N84" s="39">
+        <f>'C2 GEG Ops Budget'!L28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>Okt</t>
+        </is>
+      </c>
+      <c r="B85" s="28">
+        <f>IF(10&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!M14)</f>
+        <v/>
+      </c>
+      <c r="C85" s="28">
+        <f>'C4 GEG LR Budget'!M14</f>
+        <v/>
+      </c>
+      <c r="D85" s="28">
+        <f>IF(10&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!M86)</f>
+        <v/>
+      </c>
+      <c r="E85" s="28">
+        <f>'C4 GEG LR Budget'!M86</f>
+        <v/>
+      </c>
+      <c r="F85" s="28">
+        <f>IF(10&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!M9)</f>
+        <v/>
+      </c>
+      <c r="G85" s="28">
+        <f>'C2 GEG Ops Budget'!M9</f>
+        <v/>
+      </c>
+      <c r="H85" s="39">
+        <f>IF(10&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!M10)</f>
+        <v/>
+      </c>
+      <c r="I85" s="39">
+        <f>'C2 GEG Ops Budget'!M10</f>
+        <v/>
+      </c>
+      <c r="J85" s="39">
+        <f>IF(10&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!M25+'C5 GEG LR Aktual'!M31+'C5 GEG LR Aktual'!M41)*1000000/'C3 GEG Ops Aktual'!M19/'C3 GEG Ops Aktual'!M25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K85" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!M25+'C4 GEG LR Budget'!M31+'C4 GEG LR Budget'!M41)*1000000/'C2 GEG Ops Budget'!M19/'C2 GEG Ops Budget'!M25,NA())</f>
+        <v/>
+      </c>
+      <c r="L85" s="39">
+        <f>IF(10&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!M11+'C5 GEG LR Aktual'!M12)*1000000/'C3 GEG Ops Aktual'!M19/'C3 GEG Ops Aktual'!M25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M85" s="39">
+        <f>IF(10&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!M28)</f>
+        <v/>
+      </c>
+      <c r="N85" s="39">
+        <f>'C2 GEG Ops Budget'!M28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="B86" s="28">
+        <f>IF(11&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!N14)</f>
+        <v/>
+      </c>
+      <c r="C86" s="28">
+        <f>'C4 GEG LR Budget'!N14</f>
+        <v/>
+      </c>
+      <c r="D86" s="28">
+        <f>IF(11&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!N86)</f>
+        <v/>
+      </c>
+      <c r="E86" s="28">
+        <f>'C4 GEG LR Budget'!N86</f>
+        <v/>
+      </c>
+      <c r="F86" s="28">
+        <f>IF(11&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!N9)</f>
+        <v/>
+      </c>
+      <c r="G86" s="28">
+        <f>'C2 GEG Ops Budget'!N9</f>
+        <v/>
+      </c>
+      <c r="H86" s="39">
+        <f>IF(11&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!N10)</f>
+        <v/>
+      </c>
+      <c r="I86" s="39">
+        <f>'C2 GEG Ops Budget'!N10</f>
+        <v/>
+      </c>
+      <c r="J86" s="39">
+        <f>IF(11&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!N25+'C5 GEG LR Aktual'!N31+'C5 GEG LR Aktual'!N41)*1000000/'C3 GEG Ops Aktual'!N19/'C3 GEG Ops Aktual'!N25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K86" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!N25+'C4 GEG LR Budget'!N31+'C4 GEG LR Budget'!N41)*1000000/'C2 GEG Ops Budget'!N19/'C2 GEG Ops Budget'!N25,NA())</f>
+        <v/>
+      </c>
+      <c r="L86" s="39">
+        <f>IF(11&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!N11+'C5 GEG LR Aktual'!N12)*1000000/'C3 GEG Ops Aktual'!N19/'C3 GEG Ops Aktual'!N25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M86" s="39">
+        <f>IF(11&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!N28)</f>
+        <v/>
+      </c>
+      <c r="N86" s="39">
+        <f>'C2 GEG Ops Budget'!N28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
+        <is>
+          <t>Des</t>
+        </is>
+      </c>
+      <c r="B87" s="28">
+        <f>IF(12&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!O14)</f>
+        <v/>
+      </c>
+      <c r="C87" s="28">
+        <f>'C4 GEG LR Budget'!O14</f>
+        <v/>
+      </c>
+      <c r="D87" s="28">
+        <f>IF(12&gt;'C1 GEG Setting'!$C$6,NA(),'C5 GEG LR Aktual'!O86)</f>
+        <v/>
+      </c>
+      <c r="E87" s="28">
+        <f>'C4 GEG LR Budget'!O86</f>
+        <v/>
+      </c>
+      <c r="F87" s="28">
+        <f>IF(12&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!O9)</f>
+        <v/>
+      </c>
+      <c r="G87" s="28">
+        <f>'C2 GEG Ops Budget'!O9</f>
+        <v/>
+      </c>
+      <c r="H87" s="39">
+        <f>IF(12&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!O10)</f>
+        <v/>
+      </c>
+      <c r="I87" s="39">
+        <f>'C2 GEG Ops Budget'!O10</f>
+        <v/>
+      </c>
+      <c r="J87" s="39">
+        <f>IF(12&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!O25+'C5 GEG LR Aktual'!O31+'C5 GEG LR Aktual'!O41)*1000000/'C3 GEG Ops Aktual'!O19/'C3 GEG Ops Aktual'!O25,NA()))</f>
+        <v/>
+      </c>
+      <c r="K87" s="39">
+        <f>IFERROR(('C4 GEG LR Budget'!O25+'C4 GEG LR Budget'!O31+'C4 GEG LR Budget'!O41)*1000000/'C2 GEG Ops Budget'!O19/'C2 GEG Ops Budget'!O25,NA())</f>
+        <v/>
+      </c>
+      <c r="L87" s="39">
+        <f>IF(12&gt;'C1 GEG Setting'!$C$6,NA(),IFERROR(('C5 GEG LR Aktual'!O11+'C5 GEG LR Aktual'!O12)*1000000/'C3 GEG Ops Aktual'!O19/'C3 GEG Ops Aktual'!O25,NA()))</f>
+        <v/>
+      </c>
+      <c r="M87" s="39">
+        <f>IF(12&gt;'C1 GEG Setting'!$C$6,NA(),'C3 GEG Ops Aktual'!O28)</f>
+        <v/>
+      </c>
+      <c r="N87" s="39">
+        <f>'C2 GEG Ops Budget'!O28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>DATA GRAFIK – Struktur biaya kas YTD (Rp juta)</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="n"/>
+      <c r="C89" s="5" t="n"/>
+      <c r="D89" s="5" t="n"/>
+      <c r="E89" s="5" t="n"/>
+      <c r="F89" s="5" t="n"/>
+      <c r="G89" s="5" t="n"/>
+      <c r="H89" s="5" t="n"/>
+      <c r="I89" s="5" t="n"/>
+      <c r="J89" s="5" t="n"/>
+      <c r="K89" s="5" t="n"/>
+      <c r="L89" s="5" t="n"/>
+      <c r="M89" s="5" t="n"/>
+      <c r="N89" s="5" t="n"/>
+      <c r="O89" s="5" t="n"/>
+      <c r="P89" s="5" t="n"/>
+      <c r="Q89" s="5" t="n"/>
+      <c r="R89" s="5" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="16" t="inlineStr">
+        <is>
+          <t>Komponen</t>
+        </is>
+      </c>
+      <c r="B90" s="16" t="inlineStr">
+        <is>
+          <t>Aktual YTD</t>
+        </is>
+      </c>
+      <c r="C90" s="16" t="inlineStr">
+        <is>
+          <t>Budget YTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>Pengupasan OB</t>
+        </is>
+      </c>
+      <c r="B91" s="28">
+        <f>'C8 GEG Lap LR'!$J$16+'C8 GEG Lap LR'!$J$17+'C8 GEG Lap LR'!$J$18</f>
+        <v/>
+      </c>
+      <c r="C91" s="28">
+        <f>'C8 GEG Lap LR'!$K$16+'C8 GEG Lap LR'!$K$17+'C8 GEG Lap LR'!$K$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="inlineStr">
+        <is>
+          <t>Coal getting &amp; tambang lain</t>
+        </is>
+      </c>
+      <c r="B92" s="28">
+        <f>'C8 GEG Lap LR'!$J$19+'C8 GEG Lap LR'!$J$20+'C8 GEG Lap LR'!$J$21+'C8 GEG Lap LR'!$J$22+'C8 GEG Lap LR'!$J$23</f>
+        <v/>
+      </c>
+      <c r="C92" s="28">
+        <f>'C8 GEG Lap LR'!$K$19+'C8 GEG Lap LR'!$K$20+'C8 GEG Lap LR'!$K$21+'C8 GEG Lap LR'!$K$22+'C8 GEG Lap LR'!$K$23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t>Pengolahan &amp; hauling</t>
+        </is>
+      </c>
+      <c r="B93" s="28">
+        <f>'C8 GEG Lap LR'!$J$26+'C8 GEG Lap LR'!$J$27</f>
+        <v/>
+      </c>
+      <c r="C93" s="28">
+        <f>'C8 GEG Lap LR'!$K$26+'C8 GEG Lap LR'!$K$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="inlineStr">
+        <is>
+          <t>Pelabuhan &amp; barging</t>
+        </is>
+      </c>
+      <c r="B94" s="28">
+        <f>'C8 GEG Lap LR'!$J$28+'C8 GEG Lap LR'!$J$29</f>
+        <v/>
+      </c>
+      <c r="C94" s="28">
+        <f>'C8 GEG Lap LR'!$K$28+'C8 GEG Lap LR'!$K$29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="inlineStr">
+        <is>
+          <t>Royalti</t>
+        </is>
+      </c>
+      <c r="B95" s="28">
+        <f>'C8 GEG Lap LR'!$J$32</f>
+        <v/>
+      </c>
+      <c r="C95" s="28">
+        <f>'C8 GEG Lap LR'!$K$32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="10" t="inlineStr">
+        <is>
+          <t>Overhead site</t>
+        </is>
+      </c>
+      <c r="B96" s="28">
+        <f>'C8 GEG Lap LR'!$J$40</f>
+        <v/>
+      </c>
+      <c r="C96" s="28">
+        <f>'C8 GEG Lap LR'!$K$40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="inlineStr">
+        <is>
+          <t>Beban penjualan</t>
+        </is>
+      </c>
+      <c r="B97" s="28">
+        <f>'C8 GEG Lap LR'!$J$59</f>
+        <v/>
+      </c>
+      <c r="C97" s="28">
+        <f>'C8 GEG Lap LR'!$K$59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="10" t="inlineStr">
+        <is>
+          <t>G&amp;A excl. penyusutan</t>
+        </is>
+      </c>
+      <c r="B98" s="28">
+        <f>'C8 GEG Lap LR'!$J$70-'C8 GEG Lap LR'!$J$68</f>
+        <v/>
+      </c>
+      <c r="C98" s="28">
+        <f>'C8 GEG Lap LR'!$K$70-'C8 GEG Lap LR'!$K$68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>DATA GRAFIK – Skor KPI per perspektif &amp; jumlah status</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="n"/>
+      <c r="C100" s="5" t="n"/>
+      <c r="D100" s="5" t="n"/>
+      <c r="E100" s="5" t="n"/>
+      <c r="F100" s="5" t="n"/>
+      <c r="G100" s="5" t="n"/>
+      <c r="H100" s="5" t="n"/>
+      <c r="I100" s="5" t="n"/>
+      <c r="J100" s="5" t="n"/>
+      <c r="K100" s="5" t="n"/>
+      <c r="L100" s="5" t="n"/>
+      <c r="M100" s="5" t="n"/>
+      <c r="N100" s="5" t="n"/>
+      <c r="O100" s="5" t="n"/>
+      <c r="P100" s="5" t="n"/>
+      <c r="Q100" s="5" t="n"/>
+      <c r="R100" s="5" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="16" t="inlineStr">
+        <is>
+          <t>Perspektif</t>
+        </is>
+      </c>
+      <c r="B101" s="16" t="inlineStr">
+        <is>
+          <t>Skor rata-rata (1–5)</t>
+        </is>
+      </c>
+      <c r="C101" s="16" t="inlineStr"/>
+      <c r="D101" s="16" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E101" s="16" t="inlineStr">
+        <is>
+          <t>Jumlah KPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$47</f>
+        <v/>
+      </c>
+      <c r="B102" s="39">
+        <f>'C11 GEG KPI Scorecard'!$K$47</f>
+        <v/>
+      </c>
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>Hijau</t>
+        </is>
+      </c>
+      <c r="E102" s="28">
+        <f>'C11 GEG KPI Scorecard'!$K$44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$48</f>
+        <v/>
+      </c>
+      <c r="B103" s="39">
+        <f>'C11 GEG KPI Scorecard'!$K$48</f>
+        <v/>
+      </c>
+      <c r="D103" s="10" t="inlineStr">
+        <is>
+          <t>Kuning</t>
+        </is>
+      </c>
+      <c r="E103" s="28">
+        <f>'C11 GEG KPI Scorecard'!$L$44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$49</f>
+        <v/>
+      </c>
+      <c r="B104" s="39">
+        <f>'C11 GEG KPI Scorecard'!$K$49</f>
+        <v/>
+      </c>
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>Merah</t>
+        </is>
+      </c>
+      <c r="E104" s="28">
+        <f>'C11 GEG KPI Scorecard'!$M$44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$50</f>
+        <v/>
+      </c>
+      <c r="B105" s="39">
+        <f>'C11 GEG KPI Scorecard'!$K$50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="102">
+        <f>'C11 GEG KPI Scorecard'!$C$51</f>
+        <v/>
+      </c>
+      <c r="B106" s="39">
+        <f>'C11 GEG KPI Scorecard'!$K$51</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="24">
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="M7:O7"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="M6:O6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="M4:O4"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="M5:O5"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="P6:R6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A7">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
+      <formula>"▲ Sesuai / lebih baik dari budget"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+      <formula>"▼ Lebih buruk dari budget"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
+      <formula>"▲ Sesuai / lebih baik dari budget"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4">
+      <formula>"▼ Lebih buruk dari budget"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
+      <formula>"▲ Sesuai / lebih baik dari budget"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="4">
+      <formula>"▼ Lebih buruk dari budget"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
+      <formula>"▲ Sesuai / lebih baik dari budget"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="4">
+      <formula>"▼ Lebih buruk dari budget"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M7">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="3">
+      <formula>"▲ Sesuai / lebih baik dari budget"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="4">
+      <formula>"▼ Lebih buruk dari budget"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B76:N87">
+    <cfRule type="expression" priority="11" dxfId="5">
+      <formula>ISNA(B76)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X11:X43">
+    <cfRule type="dataBar" priority="12">
+      <dataBar showValue="1">
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="5"/>
+        <color rgb="002A78D6"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y11:Y43">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="0">
+      <formula>"Hijau"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="2">
+      <formula>"Kuning"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="1">
+      <formula>"Merah"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix overlapping chart titles and legends on GEG dashboard
Chart titles now use explicit non-overlay 11pt text, legends move below the
plot area, titles are shortened, the status tile text is compacted, and the
frozen pane that hid the KPI tiles is removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019cy6heYZTs4S4dMR3vbYtW
</commit_message>
<xml_diff>
--- a/docs/fpa-global-energy-group/GEG_FPA_Coal_Mining_Template.xlsx
+++ b/docs/fpa-global-energy-group/GEG_FPA_Coal_Mining_Template.xlsx
@@ -47,7 +47,7 @@
     <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;;(0.00&quot;x&quot;);&quot;-&quot;"/>
     <numFmt numFmtId="170" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -165,6 +165,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="0052514E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="10"/>
@@ -236,15 +241,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -366,11 +371,12 @@
     <xf numFmtId="0" fontId="18" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -521,14 +527,24 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Pendapatan bulanan: Aktual vs Budget (Rp juta)</a:t>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Pendapatan Bulanan (Rp juta)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -645,7 +661,8 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="t"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -662,14 +679,24 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>EBITDA bulanan: Aktual vs Budget (Rp juta)</a:t>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>EBITDA Bulanan (Rp juta)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -786,7 +813,8 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="t"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -803,14 +831,24 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Produksi batubara bulanan (ton)</a:t>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Produksi Batubara Bulanan (ton)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -927,7 +965,8 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="t"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -944,14 +983,24 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Stripping ratio (bcm/t): Aktual vs Budget</a:t>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Stripping Ratio (bcm/t)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -1095,7 +1144,8 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="t"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1112,14 +1162,24 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Cash cost FOB excl. royalti vs ASP (USD/t)</a:t>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cash Cost FOB vs Harga Jual (USD/t)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -1306,7 +1366,8 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="t"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1323,14 +1384,24 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Fuel ratio (L/bcm): Aktual vs Budget</a:t>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Fuel Ratio (L/bcm)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -1474,7 +1545,8 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="t"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1491,14 +1563,24 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Struktur biaya kas YTD (Rp juta)</a:t>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Struktur Biaya Kas YTD (Rp juta)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1615,7 +1697,8 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="t"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1632,14 +1715,24 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Skor KPI per perspektif (skala 1–5)</a:t>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Skor KPI per Perspektif (1–5)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1744,14 +1837,24 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:r>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t>Jumlah KPI per status</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -32079,8 +32182,8 @@
         <f>IF('C10 GEG COP'!$L$19&lt;='C10 GEG COP'!$M$19,"▲ Sesuai / lebih baik dari budget","▼ Lebih buruk dari budget")</f>
         <v/>
       </c>
-      <c r="P7" s="96">
-        <f>"Hijau "&amp;'C11 GEG KPI Scorecard'!$K$44&amp;" | Kuning "&amp;'C11 GEG KPI Scorecard'!$L$44&amp;" | Merah "&amp;'C11 GEG KPI Scorecard'!$M$44</f>
+      <c r="P7" s="99">
+        <f>"Hijau "&amp;'C11 GEG KPI Scorecard'!$K$44&amp;" · Kuning "&amp;'C11 GEG KPI Scorecard'!$L$44&amp;" · Merah "&amp;'C11 GEG KPI Scorecard'!$M$44</f>
         <v/>
       </c>
     </row>
@@ -32107,7 +32210,7 @@
       <c r="P9" s="5" t="n"/>
       <c r="Q9" s="5" t="n"/>
       <c r="R9" s="5" t="n"/>
-      <c r="S9" s="99" t="inlineStr">
+      <c r="S9" s="100" t="inlineStr">
         <is>
           <t>KPI SCORED – YTD</t>
         </is>
@@ -32120,44 +32223,44 @@
       <c r="Y9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="S10" s="100" t="inlineStr">
+      <c r="S10" s="101" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="T10" s="100" t="inlineStr">
+      <c r="T10" s="101" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="U10" s="100" t="inlineStr">
+      <c r="U10" s="101" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="V10" s="100" t="inlineStr">
+      <c r="V10" s="101" t="inlineStr">
         <is>
           <t>Aktual</t>
         </is>
       </c>
-      <c r="W10" s="100" t="inlineStr">
+      <c r="W10" s="101" t="inlineStr">
         <is>
           <t>Pencapaian</t>
         </is>
       </c>
-      <c r="X10" s="100" t="inlineStr">
+      <c r="X10" s="101" t="inlineStr">
         <is>
           <t>Skor</t>
         </is>
       </c>
-      <c r="Y10" s="100" t="inlineStr">
+      <c r="Y10" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="S11" s="101">
+      <c r="S11" s="102">
         <f>'C11 GEG KPI Scorecard'!$A$6</f>
         <v/>
       </c>
@@ -32173,7 +32276,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$7</f>
         <v/>
       </c>
-      <c r="T12" s="102">
+      <c r="T12" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$7</f>
         <v/>
       </c>
@@ -32203,7 +32306,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$8</f>
         <v/>
       </c>
-      <c r="T13" s="102">
+      <c r="T13" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$8</f>
         <v/>
       </c>
@@ -32233,7 +32336,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$9</f>
         <v/>
       </c>
-      <c r="T14" s="102">
+      <c r="T14" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$9</f>
         <v/>
       </c>
@@ -32263,7 +32366,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$10</f>
         <v/>
       </c>
-      <c r="T15" s="102">
+      <c r="T15" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$10</f>
         <v/>
       </c>
@@ -32293,7 +32396,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$11</f>
         <v/>
       </c>
-      <c r="T16" s="102">
+      <c r="T16" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$11</f>
         <v/>
       </c>
@@ -32323,7 +32426,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$12</f>
         <v/>
       </c>
-      <c r="T17" s="102">
+      <c r="T17" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$12</f>
         <v/>
       </c>
@@ -32349,7 +32452,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="S18" s="101">
+      <c r="S18" s="102">
         <f>'C11 GEG KPI Scorecard'!$A$13</f>
         <v/>
       </c>
@@ -32365,7 +32468,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$14</f>
         <v/>
       </c>
-      <c r="T19" s="102">
+      <c r="T19" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$14</f>
         <v/>
       </c>
@@ -32395,7 +32498,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$15</f>
         <v/>
       </c>
-      <c r="T20" s="102">
+      <c r="T20" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$15</f>
         <v/>
       </c>
@@ -32425,7 +32528,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$16</f>
         <v/>
       </c>
-      <c r="T21" s="102">
+      <c r="T21" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$16</f>
         <v/>
       </c>
@@ -32455,7 +32558,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$17</f>
         <v/>
       </c>
-      <c r="T22" s="102">
+      <c r="T22" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$17</f>
         <v/>
       </c>
@@ -32485,7 +32588,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$18</f>
         <v/>
       </c>
-      <c r="T23" s="102">
+      <c r="T23" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$18</f>
         <v/>
       </c>
@@ -32515,7 +32618,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$19</f>
         <v/>
       </c>
-      <c r="T24" s="102">
+      <c r="T24" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$19</f>
         <v/>
       </c>
@@ -32541,7 +32644,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="S25" s="101">
+      <c r="S25" s="102">
         <f>'C11 GEG KPI Scorecard'!$A$20</f>
         <v/>
       </c>
@@ -32557,7 +32660,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$21</f>
         <v/>
       </c>
-      <c r="T26" s="102">
+      <c r="T26" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$21</f>
         <v/>
       </c>
@@ -32587,7 +32690,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$22</f>
         <v/>
       </c>
-      <c r="T27" s="102">
+      <c r="T27" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$22</f>
         <v/>
       </c>
@@ -32617,7 +32720,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$23</f>
         <v/>
       </c>
-      <c r="T28" s="102">
+      <c r="T28" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$23</f>
         <v/>
       </c>
@@ -32647,7 +32750,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$24</f>
         <v/>
       </c>
-      <c r="T29" s="102">
+      <c r="T29" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$24</f>
         <v/>
       </c>
@@ -32677,7 +32780,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$25</f>
         <v/>
       </c>
-      <c r="T30" s="102">
+      <c r="T30" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$25</f>
         <v/>
       </c>
@@ -32703,7 +32806,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="S31" s="101">
+      <c r="S31" s="102">
         <f>'C11 GEG KPI Scorecard'!$A$26</f>
         <v/>
       </c>
@@ -32719,7 +32822,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$27</f>
         <v/>
       </c>
-      <c r="T32" s="102">
+      <c r="T32" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$27</f>
         <v/>
       </c>
@@ -32749,7 +32852,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$28</f>
         <v/>
       </c>
-      <c r="T33" s="102">
+      <c r="T33" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$28</f>
         <v/>
       </c>
@@ -32779,7 +32882,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$29</f>
         <v/>
       </c>
-      <c r="T34" s="102">
+      <c r="T34" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$29</f>
         <v/>
       </c>
@@ -32809,7 +32912,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$30</f>
         <v/>
       </c>
-      <c r="T35" s="102">
+      <c r="T35" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$30</f>
         <v/>
       </c>
@@ -32839,7 +32942,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$31</f>
         <v/>
       </c>
-      <c r="T36" s="102">
+      <c r="T36" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$31</f>
         <v/>
       </c>
@@ -32869,7 +32972,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$32</f>
         <v/>
       </c>
-      <c r="T37" s="102">
+      <c r="T37" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$32</f>
         <v/>
       </c>
@@ -32895,7 +32998,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="S38" s="101">
+      <c r="S38" s="102">
         <f>'C11 GEG KPI Scorecard'!$A$33</f>
         <v/>
       </c>
@@ -32911,7 +33014,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$34</f>
         <v/>
       </c>
-      <c r="T39" s="102">
+      <c r="T39" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$34</f>
         <v/>
       </c>
@@ -32941,7 +33044,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$35</f>
         <v/>
       </c>
-      <c r="T40" s="102">
+      <c r="T40" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$35</f>
         <v/>
       </c>
@@ -32971,7 +33074,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$36</f>
         <v/>
       </c>
-      <c r="T41" s="102">
+      <c r="T41" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$36</f>
         <v/>
       </c>
@@ -33001,7 +33104,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$37</f>
         <v/>
       </c>
-      <c r="T42" s="102">
+      <c r="T42" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$37</f>
         <v/>
       </c>
@@ -33031,7 +33134,7 @@
         <f>'C11 GEG KPI Scorecard'!$A$38</f>
         <v/>
       </c>
-      <c r="T43" s="102">
+      <c r="T43" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$38</f>
         <v/>
       </c>
@@ -33062,11 +33165,11 @@
           <t>SKOR TERTIMBANG TOTAL</t>
         </is>
       </c>
-      <c r="X44" s="103">
+      <c r="X44" s="104">
         <f>'C11 GEG KPI Scorecard'!$L$42</f>
         <v/>
       </c>
-      <c r="Y44" s="104">
+      <c r="Y44" s="105">
         <f>'C11 GEG KPI Scorecard'!$L$43</f>
         <v/>
       </c>
@@ -34091,7 +34194,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="102">
+      <c r="A102" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$47</f>
         <v/>
       </c>
@@ -34110,7 +34213,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="102">
+      <c r="A103" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$48</f>
         <v/>
       </c>
@@ -34129,7 +34232,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="102">
+      <c r="A104" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$49</f>
         <v/>
       </c>
@@ -34148,7 +34251,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="102">
+      <c r="A105" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$50</f>
         <v/>
       </c>
@@ -34158,7 +34261,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="102">
+      <c r="A106" s="103">
         <f>'C11 GEG KPI Scorecard'!$C$51</f>
         <v/>
       </c>

</xml_diff>